<commit_message>
Committing again before making possibly breaking changes.
</commit_message>
<xml_diff>
--- a/DocumentProcessor.Avalonia.TerrenceLGee/contacts.xlsx
+++ b/DocumentProcessor.Avalonia.TerrenceLGee/contacts.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="ContactsSheet" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,25 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="93">
-  <si>
-    <t xml:space="preserve">Id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">First Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Middle Initial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email Address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phone Number</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="87">
   <si>
     <t xml:space="preserve">Homer</t>
   </si>
@@ -313,7 +295,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -385,11 +366,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -516,401 +497,360 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.44"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.72"/>
-  </cols>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="2" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="C4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="2" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="2" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="2" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="B7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="1" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="2" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="2" t="s">
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="2" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F11" s="2" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="2" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="B13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="2" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="B14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2" t="s">
+      <c r="D14" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="2" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="B15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="2" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="B16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="2" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="B17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="2" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F18" s="1" t="s">
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="B20" s="2"/>
+      <c r="C20" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="D20" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="1" t="s">
+      <c r="E20" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="1" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="B21" s="2"/>
+      <c r="C21" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="1" t="s">
+      <c r="D21" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>